<commit_message>
docs: restyle UI review checklist
</commit_message>
<xml_diff>
--- a/UI-UX/docs/ui-v1-review-2026-04-28.xlsx
+++ b/UI-UX/docs/ui-v1-review-2026-04-28.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,8 +80,46 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00155E63"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00164E63"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="001F2937"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007E22CE"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00164E63"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -128,8 +166,38 @@
         <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDF7F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFFAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F2FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -165,11 +233,39 @@
         <color rgb="007C93A0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="medium">
+        <color rgb="005B8790"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -236,6 +332,87 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -605,1243 +782,1243 @@
   <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="27" customHeight="1">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Review UI v1: проверка по ТЗ</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Принцип: сначала проверяем требования ТЗ, затем отдельным блоком добавляем замечания вне ТЗ как «Доп. UI/UX». Лишние backend-only пункты убраны.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Раздел ТЗ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>Требование / вопрос</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>Где смотреть в UI</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="25" t="inlineStr">
         <is>
           <t>Что проверить</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="25" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="25" t="inlineStr">
         <is>
           <t>Комментарий участника</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="25" t="inlineStr">
         <is>
           <t>Комментарий заказчика</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="25" t="inlineStr">
         <is>
           <t>Действие</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="5" ht="68" customHeight="1">
+      <c r="A5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>1.2 / 7.2</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="29" t="inlineStr">
         <is>
           <t>ИИ не принимает инженерное решение. Инженер должен видеть основания и сам принимать финальное решение.</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="29" t="inlineStr">
         <is>
           <t>Чат, Проверка</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="29" t="inlineStr">
         <is>
           <t>Нет ли формулировок, будто система сама принимает решение. Понятно ли, что ответ основан на документах.</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr"/>
-      <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H5" s="29" t="inlineStr"/>
+      <c r="I5" s="29" t="inlineStr"/>
+      <c r="J5" s="29" t="inlineStr">
         <is>
           <t>Проверить тексты ответов и статусов.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="8" t="n">
+    <row r="6" ht="68" customHeight="1">
+      <c r="A6" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>1.2 / 3.4 / 7.2</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>Ответ всегда сопровождается источником: документом и фрагментом.</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="32" t="inlineStr">
         <is>
           <t>Чат</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="32" t="inlineStr">
         <is>
           <t>У каждого пункта ответа есть ссылки «Страница» и «Документ». Ссылки открываются справа.</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H6" s="32" t="inlineStr"/>
+      <c r="I6" s="32" t="inlineStr"/>
+      <c r="J6" s="32" t="inlineStr">
         <is>
           <t>Отметить ответы без источников.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="7" ht="68" customHeight="1">
+      <c r="A7" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="28" t="inlineStr">
         <is>
           <t>1.2 / 3.5</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>Если данных недостаточно, система должна уточнить запрос.</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>Чат</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="29" t="inlineStr">
         <is>
           <t>Понятно ли, как UI показывает уточняющий вопрос или нехватку данных.</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="33" t="inlineStr">
         <is>
           <t>Уточнить</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="H7" s="29" t="inlineStr"/>
+      <c r="I7" s="29" t="inlineStr"/>
+      <c r="J7" s="29" t="inlineStr">
         <is>
           <t>Согласовать с backend формат такого ответа.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="8" t="n">
+    <row r="8" ht="68" customHeight="1">
+      <c r="A8" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>1.1 / 7.2</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>One-shot сценарий: инженер задает вопрос и быстро получает ответ.</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="32" t="inlineStr">
         <is>
           <t>Чат</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="32" t="inlineStr">
         <is>
           <t>Поле ввода видно сразу. Ответ, источники и статус не требуют лишних переходов.</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H8" s="32" t="inlineStr"/>
+      <c r="I8" s="32" t="inlineStr"/>
+      <c r="J8" s="32" t="inlineStr">
         <is>
           <t>Проверить основной сценарий на демо.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
-      <c r="A9" s="4" t="n">
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="28" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>Поиск по базе знаний НСИ: выдача документов, фрагментов и релевантности.</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>Поиск</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="29" t="inlineStr">
         <is>
           <t>Понятна ли поисковая выдача. Можно ли открыть страницу и документ.</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="inlineStr"/>
+      <c r="I9" s="29" t="inlineStr"/>
+      <c r="J9" s="29" t="inlineStr">
         <is>
           <t>Проверить несколько запросов.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
-      <c r="A10" s="8" t="n">
+    <row r="10" ht="68" customHeight="1">
+      <c r="A10" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>Диалоговый режим: пользователь должен отличать свой запрос от ответа ассистента.</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="32" t="inlineStr">
         <is>
           <t>Чат</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="32" t="inlineStr">
         <is>
           <t>Запрос инженера и ответ ассистента визуально различаются, но не перегружают экран.</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr">
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H10" s="32" t="inlineStr"/>
+      <c r="I10" s="32" t="inlineStr"/>
+      <c r="J10" s="32" t="inlineStr">
         <is>
           <t>Оценить читаемость диалога.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="54" customHeight="1">
-      <c r="A11" s="4" t="n">
+    <row r="11" ht="68" customHeight="1">
+      <c r="A11" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="28" t="inlineStr">
         <is>
           <t>3.9</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="29" t="inlineStr">
         <is>
           <t>История должна хранить запрос, ответ, пользователя и источники.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>История</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="29" t="inlineStr">
         <is>
           <t>В таблице истории есть нужные поля, фильтры и переход к источникам.</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
-      <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="inlineStr"/>
+      <c r="I11" s="29" t="inlineStr"/>
+      <c r="J11" s="29" t="inlineStr">
         <is>
           <t>Отметить недостающие поля.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="8" t="n">
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>3.9</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>История должна поддерживать поиск, аналитику и экспорт.</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>История</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="32" t="inlineStr">
         <is>
           <t>Фильтры работают понятно. Экспорт учитывает текущую выборку.</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr">
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H12" s="32" t="inlineStr"/>
+      <c r="I12" s="32" t="inlineStr"/>
+      <c r="J12" s="32" t="inlineStr">
         <is>
           <t>Проверить экспорт после фильтрации.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="4" t="n">
+    <row r="13" ht="68" customHeight="1">
+      <c r="A13" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="28" t="inlineStr">
         <is>
           <t>3.1 / 7.1</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>Администрирование базы НСИ: загрузка и управление документами.</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>Реестр, Администрирование</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="29" t="inlineStr">
         <is>
           <t>Есть ли понятная загрузка документов, список документов и действия по обновлению.</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="inlineStr"/>
+      <c r="I13" s="29" t="inlineStr"/>
+      <c r="J13" s="29" t="inlineStr">
         <is>
           <t>Уточнить, какие действия нужны администратору знаний.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="54" customHeight="1">
-      <c r="A14" s="8" t="n">
+    <row r="14" ht="68" customHeight="1">
+      <c r="A14" s="30" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>OCR и извлечение данных должны быть видны через статусы обработки.</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="32" t="inlineStr">
         <is>
           <t>Реестр, QA</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="32" t="inlineStr">
         <is>
           <t>Показываются ли OCR-статусы, ошибки, проблемные документы и переобработка.</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr"/>
-      <c r="I14" s="9" t="inlineStr"/>
-      <c r="J14" s="9" t="inlineStr">
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H14" s="32" t="inlineStr"/>
+      <c r="I14" s="32" t="inlineStr"/>
+      <c r="J14" s="32" t="inlineStr">
         <is>
           <t>Проверить понятность OCR-статусов.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="54" customHeight="1">
-      <c r="A15" s="4" t="n">
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="28" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="29" t="inlineStr">
         <is>
           <t>База знаний: chunking, embeddings, метаданные, обновление индекса.</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="29" t="inlineStr">
         <is>
           <t>Реестр, QA</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="29" t="inlineStr">
         <is>
           <t>Видно ли, что документ обработан, индексирован и готов к поиску.</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr"/>
-      <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="inlineStr"/>
+      <c r="I15" s="29" t="inlineStr"/>
+      <c r="J15" s="29" t="inlineStr">
         <is>
           <t>Проверить статусы индексации.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="54" customHeight="1">
-      <c r="A16" s="8" t="n">
+    <row r="16" ht="68" customHeight="1">
+      <c r="A16" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>3.6</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="32" t="inlineStr">
         <is>
           <t>Проверка проектных решений на соответствие требованиям НСИ.</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="32" t="inlineStr">
         <is>
           <t>Проверка</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="32" t="inlineStr">
         <is>
           <t>Можно выбрать один или несколько документов и запустить проверку.</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr"/>
-      <c r="J16" s="9" t="inlineStr">
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H16" s="32" t="inlineStr"/>
+      <c r="I16" s="32" t="inlineStr"/>
+      <c r="J16" s="32" t="inlineStr">
         <is>
           <t>Проверить выборочную и пакетную проверку.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="54" customHeight="1">
-      <c r="A17" s="4" t="n">
+    <row r="17" ht="68" customHeight="1">
+      <c r="A17" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="28" t="inlineStr">
         <is>
           <t>3.6</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="29" t="inlineStr">
         <is>
           <t>Результат проверки должен иметь статусы OK / WARNING / ERROR.</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="29" t="inlineStr">
         <is>
           <t>Проверка</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="29" t="inlineStr">
         <is>
           <t>В таблице понятны проект, раздел, параметр, значение, требование НСИ, статус и комментарий.</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="inlineStr"/>
+      <c r="I17" s="29" t="inlineStr"/>
+      <c r="J17" s="29" t="inlineStr">
         <is>
           <t>Отметить лишние или недостающие колонки.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="54" customHeight="1">
-      <c r="A18" s="8" t="n">
+    <row r="18" ht="68" customHeight="1">
+      <c r="A18" s="30" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>3.7</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="32" t="inlineStr">
         <is>
           <t>Рекомендации: конфликты, альтернативы, смежные системы.</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="32" t="inlineStr">
         <is>
           <t>Чат, Проверка</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="32" t="inlineStr">
         <is>
           <t>Есть ли место, где UI может показать конфликт или альтернативу. Если нет — это вопрос к MVP.</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="33" t="inlineStr">
         <is>
           <t>Уточнить</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr"/>
-      <c r="I18" s="9" t="inlineStr"/>
-      <c r="J18" s="9" t="inlineStr">
+      <c r="H18" s="32" t="inlineStr"/>
+      <c r="I18" s="32" t="inlineStr"/>
+      <c r="J18" s="32" t="inlineStr">
         <is>
           <t>Решить, нужен ли отдельный блок рекомендаций.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="54" customHeight="1">
-      <c r="A19" s="4" t="n">
+    <row r="19" ht="68" customHeight="1">
+      <c r="A19" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="28" t="inlineStr">
         <is>
           <t>3.8</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="29" t="inlineStr">
         <is>
           <t>Расчетный модуль: перерасчет параметров по методикам НСИ.</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="29" t="inlineStr">
         <is>
           <t>Нет отдельного экрана</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="29" t="inlineStr">
         <is>
           <t>Нужен ли UI для расчета в первой версии или это следующий этап.</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="33" t="inlineStr">
         <is>
           <t>Уточнить</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="H19" s="29" t="inlineStr"/>
+      <c r="I19" s="29" t="inlineStr"/>
+      <c r="J19" s="29" t="inlineStr">
         <is>
           <t>Уточнить с заказчиком и техлидами.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="54" customHeight="1">
-      <c r="A20" s="8" t="n">
+    <row r="20" ht="68" customHeight="1">
+      <c r="A20" s="30" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>3.10</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="32" t="inlineStr">
         <is>
           <t>Интеграция с ИС «Меридиан»: получение данных, запись результатов, история.</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="32" t="inlineStr">
         <is>
           <t>Администрирование, QA</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="32" t="inlineStr">
         <is>
           <t>Нужно ли показывать в UI статус подключения/синхронизации с Меридианом.</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="33" t="inlineStr">
         <is>
           <t>Уточнить</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr"/>
-      <c r="I20" s="9" t="inlineStr"/>
-      <c r="J20" s="9" t="inlineStr">
+      <c r="H20" s="32" t="inlineStr"/>
+      <c r="I20" s="32" t="inlineStr"/>
+      <c r="J20" s="32" t="inlineStr">
         <is>
           <t>Уточнить, требуется ли отдельный индикатор.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="54" customHeight="1">
-      <c r="A21" s="4" t="n">
+    <row r="21" ht="68" customHeight="1">
+      <c r="A21" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="28" t="inlineStr">
         <is>
           <t>4 / 8</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="29" t="inlineStr">
         <is>
           <t>Критерии приемки: скорость, точность ответов, OCR, источники.</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="29" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="29" t="inlineStr">
         <is>
           <t>QA-вкладка показывает ключевые метрики и понятно объясняет, что они означают.</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H21" s="29" t="inlineStr"/>
+      <c r="I21" s="29" t="inlineStr"/>
+      <c r="J21" s="29" t="inlineStr">
         <is>
           <t>Сверить метрики с backend и приемкой.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="54" customHeight="1">
-      <c r="A22" s="8" t="n">
+    <row r="22" ht="68" customHeight="1">
+      <c r="A22" s="30" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="31" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="32" t="inlineStr">
         <is>
           <t>Frontend: React, TypeScript, Ant Design / shadcn.</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E22" s="32" t="inlineStr">
         <is>
           <t>README, код</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F22" s="32" t="inlineStr">
         <is>
           <t>Фактический стек указан честно. Если UI на другой библиотеке — это отмечено.</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr"/>
-      <c r="I22" s="9" t="inlineStr"/>
-      <c r="J22" s="9" t="inlineStr">
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H22" s="32" t="inlineStr"/>
+      <c r="I22" s="32" t="inlineStr"/>
+      <c r="J22" s="32" t="inlineStr">
         <is>
           <t>Записать фактическую библиотеку текущей версии.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="54" customHeight="1">
-      <c r="A23" s="4" t="n">
+    <row r="23" ht="68" customHeight="1">
+      <c r="A23" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="28" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="29" t="inlineStr">
         <is>
           <t>Основные экраны: ввод запроса, ответ с источниками, диалог, история, администрирование.</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="29" t="inlineStr">
         <is>
           <t>Навигация</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="29" t="inlineStr">
         <is>
           <t>Все обязательные экраны есть в меню и названы понятно для инженера.</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr"/>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="inlineStr"/>
+      <c r="I23" s="29" t="inlineStr"/>
+      <c r="J23" s="29" t="inlineStr">
         <is>
           <t>Проверить названия вкладок.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="54" customHeight="1">
-      <c r="A24" s="8" t="n">
+    <row r="24" ht="68" customHeight="1">
+      <c r="A24" s="30" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="32" t="inlineStr">
         <is>
           <t>Поставка: Git-репозиторий, docker-compose, README, запуск для проверки.</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E24" s="32" t="inlineStr">
         <is>
           <t>GitHub, README, Docker</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F24" s="32" t="inlineStr">
         <is>
           <t>Команда может забрать проект, запустить UI и проверить сценарии локально.</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="inlineStr"/>
-      <c r="I24" s="9" t="inlineStr"/>
-      <c r="J24" s="9" t="inlineStr">
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H24" s="32" t="inlineStr"/>
+      <c r="I24" s="32" t="inlineStr"/>
+      <c r="J24" s="32" t="inlineStr">
         <is>
           <t>Проверить инструкцию первого запуска.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="54" customHeight="1">
-      <c r="A25" s="11" t="n">
+    <row r="25" ht="68" customHeight="1">
+      <c r="A25" s="34" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C25" s="36" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D25" s="37" t="inlineStr">
         <is>
           <t>Читаемость и визуальная нагрузка.</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="37" t="inlineStr">
         <is>
           <t>Все вкладки</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F25" s="37" t="inlineStr">
         <is>
           <t>Основная функция вкладки видна сразу. Нет лишней пестроты, таблицы и чат читаются спокойно.</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr"/>
-      <c r="I25" s="13" t="inlineStr"/>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="G25" s="38" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H25" s="37" t="inlineStr"/>
+      <c r="I25" s="37" t="inlineStr"/>
+      <c r="J25" s="37" t="inlineStr">
         <is>
           <t>Собрать замечания команды по визуалу.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="54" customHeight="1">
-      <c r="A26" s="15" t="n">
+    <row r="26" ht="68" customHeight="1">
+      <c r="A26" s="30" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C26" s="16" t="inlineStr">
+      <c r="C26" s="31" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr">
+      <c r="D26" s="32" t="inlineStr">
         <is>
           <t>Единый стиль ссылок, таблиц, кнопок и статусов.</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="32" t="inlineStr">
         <is>
           <t>Чат, Поиск, Проверка, История, Реестр</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F26" s="32" t="inlineStr">
         <is>
           <t>Одинаковые сущности выглядят одинаково: «Страница», «Документ», статусы, таблицы, кнопки.</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H26" s="16" t="inlineStr"/>
-      <c r="I26" s="16" t="inlineStr"/>
-      <c r="J26" s="16" t="inlineStr">
+      <c r="G26" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H26" s="32" t="inlineStr"/>
+      <c r="I26" s="32" t="inlineStr"/>
+      <c r="J26" s="32" t="inlineStr">
         <is>
           <t>Отметить визуальный разнобой.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="54" customHeight="1">
-      <c r="A27" s="11" t="n">
+    <row r="27" ht="68" customHeight="1">
+      <c r="A27" s="26" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C27" s="28" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D27" s="29" t="inlineStr">
         <is>
           <t>Правое превью страницы и полного документа.</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E27" s="29" t="inlineStr">
         <is>
           <t>Чат, Поиск, Проверка</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="F27" s="29" t="inlineStr">
         <is>
           <t>Страница открывает конкретный фрагмент. Документ открывается полностью и удобно скроллится.</t>
         </is>
       </c>
-      <c r="G27" s="14" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H27" s="13" t="inlineStr"/>
-      <c r="I27" s="13" t="inlineStr"/>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="G27" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="inlineStr"/>
+      <c r="I27" s="29" t="inlineStr"/>
+      <c r="J27" s="29" t="inlineStr">
         <is>
           <t>Проверить удобство панели предпросмотра.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="54" customHeight="1">
-      <c r="A28" s="15" t="n">
+    <row r="28" ht="68" customHeight="1">
+      <c r="A28" s="30" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C28" s="31" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="D28" s="32" t="inlineStr">
         <is>
           <t>Фокус-режим.</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E28" s="32" t="inlineStr">
         <is>
           <t>Все вкладки</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F28" s="32" t="inlineStr">
         <is>
           <t>Фокус-режим скрывает левую панель и работает на каждой вкладке.</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H28" s="16" t="inlineStr"/>
-      <c r="I28" s="16" t="inlineStr"/>
-      <c r="J28" s="16" t="inlineStr">
+      <c r="G28" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H28" s="32" t="inlineStr"/>
+      <c r="I28" s="32" t="inlineStr"/>
+      <c r="J28" s="32" t="inlineStr">
         <is>
           <t>Проверить, не ломается ли сценарий.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="54" customHeight="1">
-      <c r="A29" s="11" t="n">
+    <row r="29" ht="68" customHeight="1">
+      <c r="A29" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C29" s="28" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="D29" s="29" t="inlineStr">
         <is>
           <t>Видеоинструкция.</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E29" s="29" t="inlineStr">
         <is>
           <t>Верхняя панель / сервисные функции</t>
         </is>
       </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="F29" s="29" t="inlineStr">
         <is>
           <t>Видеоинструкция открывается и помогает быстро понять интерфейс.</t>
         </is>
       </c>
-      <c r="G29" s="14" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="inlineStr"/>
-      <c r="I29" s="13" t="inlineStr"/>
-      <c r="J29" s="13" t="inlineStr">
+      <c r="G29" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="inlineStr"/>
+      <c r="I29" s="29" t="inlineStr"/>
+      <c r="J29" s="29" t="inlineStr">
         <is>
           <t>Проверить актуальность видео к текущей версии UI.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="17" t="n">
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="40" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="19" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="17" t="n"/>
-      <c r="J30" s="17" t="n"/>
-    </row>
-    <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="17" t="n">
+      <c r="C30" s="41" t="n"/>
+      <c r="D30" s="42" t="n"/>
+      <c r="E30" s="42" t="n"/>
+      <c r="F30" s="42" t="n"/>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H30" s="42" t="n"/>
+      <c r="I30" s="42" t="n"/>
+      <c r="J30" s="42" t="n"/>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="43" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C31" s="17" t="n"/>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
-      <c r="G31" s="19" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="17" t="n"/>
-      <c r="J31" s="17" t="n"/>
-    </row>
-    <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="17" t="n">
+      <c r="C31" s="44" t="n"/>
+      <c r="D31" s="45" t="n"/>
+      <c r="E31" s="45" t="n"/>
+      <c r="F31" s="45" t="n"/>
+      <c r="G31" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H31" s="45" t="n"/>
+      <c r="I31" s="45" t="n"/>
+      <c r="J31" s="45" t="n"/>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="40" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B32" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="17" t="n"/>
-      <c r="E32" s="17" t="n"/>
-      <c r="F32" s="17" t="n"/>
-      <c r="G32" s="19" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H32" s="17" t="n"/>
-      <c r="I32" s="17" t="n"/>
-      <c r="J32" s="17" t="n"/>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="17" t="n">
+      <c r="C32" s="41" t="n"/>
+      <c r="D32" s="42" t="n"/>
+      <c r="E32" s="42" t="n"/>
+      <c r="F32" s="42" t="n"/>
+      <c r="G32" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H32" s="42" t="n"/>
+      <c r="I32" s="42" t="n"/>
+      <c r="J32" s="42" t="n"/>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="43" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B33" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="19" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H33" s="17" t="n"/>
-      <c r="I33" s="17" t="n"/>
-      <c r="J33" s="17" t="n"/>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="17" t="n">
+      <c r="C33" s="44" t="n"/>
+      <c r="D33" s="45" t="n"/>
+      <c r="E33" s="45" t="n"/>
+      <c r="F33" s="45" t="n"/>
+      <c r="G33" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H33" s="45" t="n"/>
+      <c r="I33" s="45" t="n"/>
+      <c r="J33" s="45" t="n"/>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B34" s="39" t="inlineStr">
         <is>
           <t>Доп. UI/UX</t>
         </is>
       </c>
-      <c r="C34" s="17" t="n"/>
-      <c r="D34" s="17" t="n"/>
-      <c r="E34" s="17" t="n"/>
-      <c r="F34" s="17" t="n"/>
-      <c r="G34" s="19" t="inlineStr">
-        <is>
-          <t>Не проверено</t>
-        </is>
-      </c>
-      <c r="H34" s="17" t="n"/>
-      <c r="I34" s="17" t="n"/>
-      <c r="J34" s="17" t="n"/>
+      <c r="C34" s="41" t="n"/>
+      <c r="D34" s="42" t="n"/>
+      <c r="E34" s="42" t="n"/>
+      <c r="F34" s="42" t="n"/>
+      <c r="G34" s="27" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="H34" s="42" t="n"/>
+      <c r="I34" s="42" t="n"/>
+      <c r="J34" s="42" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:J34"/>
@@ -1850,10 +2027,10 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="G5:G79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Не проверено,ОК,Доработать,Уточнить"</formula1>
+    <dataValidation sqref="G5:G84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Проверить,ОК,Доработать,Уточнить"</formula1>
     </dataValidation>
-    <dataValidation sqref="B5:B79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B5:B84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ТЗ,Доп. UI/UX"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1870,168 +2047,185 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="61" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>Как заполнять review</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Поле</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Что писать</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Пример</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
-        <is>
-          <t>ТЗ — требование заказчика. Доп. UI/UX — наша инициатива, визуал, удобство, демо-сценарий.</t>
-        </is>
-      </c>
-      <c r="C4" s="22" t="inlineStr">
+      <c r="B3" s="47" t="inlineStr">
+        <is>
+          <t>ТЗ — требование заказчика. Доп. UI/UX — наша инициатива: визуал, удобство, демо-сценарий.</t>
+        </is>
+      </c>
+      <c r="C3" s="47" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Раздел ТЗ</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>Номер раздела из технического задания. Для доп. UI/UX можно ставить «-».</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Номер раздела из технического задания. Если смысл есть в нескольких местах, писать через слэш.</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>1.2 / 3.4 / 7.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Требование / вопрос</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>Коротко: что должно быть или что надо решить.</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Коротко: что должно быть в UI или какой вопрос надо решить.</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
         <is>
           <t>Ответ должен иметь источник.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="48" t="inlineStr">
         <is>
           <t>Где смотреть в UI</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B6" s="48" t="inlineStr">
         <is>
           <t>Вкладка или зона интерфейса.</t>
         </is>
       </c>
-      <c r="C7" s="22" t="inlineStr">
+      <c r="C6" s="48" t="inlineStr">
         <is>
           <t>Чат</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>Что проверить</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
-        <is>
-          <t>Конкретное действие тестировщика/участника.</t>
-        </is>
-      </c>
-      <c r="C8" s="22" t="inlineStr">
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Конкретное действие проверяющего.</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
         <is>
           <t>Открыть страницу и документ справа.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="48" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
-        <is>
-          <t>Не проверено, ОК, Доработать или Уточнить.</t>
-        </is>
-      </c>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>Проверить — еще не смотрели; ОК — все нормально; Доработать — нужна правка; Уточнить — нужен вопрос заказчику, backend или тимлиду.</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
         <is>
           <t>Уточнить</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>Комментарий участника</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B9" s="49" t="inlineStr">
         <is>
           <t>Что заметил человек после запуска.</t>
         </is>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
           <t>Ссылка на документ неочевидна.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="48" t="inlineStr">
         <is>
           <t>Комментарий заказчика</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>Что сказал заказчик после показа.</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C10" s="48" t="inlineStr">
         <is>
           <t>Просит добавить статус Меридиана.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>Действие</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Что сделать дальше. Если статус «Уточнить», здесь пишем у кого и что уточнить.</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="inlineStr">
+        <is>
+          <t>Уточнить у backend формат ответа без данных.</t>
         </is>
       </c>
     </row>

</xml_diff>